<commit_message>
Add sync_orchestrator.py: chains stub_detector + workbook_bridge, embeds tasks into agent_orchestrator.html, wired into pre-commit
</commit_message>
<xml_diff>
--- a/Semptify_Master_Inventory_LIVE_reviewed.xlsx
+++ b/Semptify_Master_Inventory_LIVE_reviewed.xlsx
@@ -2399,7 +2399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F156"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="24" min="1" max="1"/>
@@ -2442,4656 +2442,161 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1" s="25">
-      <c r="A2" s="35" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="35" t="inlineStr">
-        <is>
-          <t>case_builder.py</t>
-        </is>
-      </c>
-      <c r="C2" s="35" t="inlineStr">
-        <is>
-          <t>860</t>
-        </is>
-      </c>
-      <c r="D2" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E2" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F2" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="15" customHeight="1" s="25">
-      <c r="A3" s="33" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="33" t="inlineStr">
-        <is>
-          <t>complaint_wizard_module.py</t>
-        </is>
-      </c>
-      <c r="C3" s="33" t="inlineStr">
-        <is>
-          <t>444</t>
-        </is>
-      </c>
-      <c r="D3" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E3" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F3" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1" s="25">
-      <c r="A4" s="35" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="35" t="inlineStr">
-        <is>
-          <t>complaint_wizard_module.py</t>
-        </is>
-      </c>
-      <c r="C4" s="35" t="inlineStr">
-        <is>
-          <t>618</t>
-        </is>
-      </c>
-      <c r="D4" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E4" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F4" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="25">
-      <c r="A5" s="34" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="34" t="inlineStr">
-        <is>
-          <t>legal_filing_module.py</t>
-        </is>
-      </c>
-      <c r="C5" s="34" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="D5" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E5" s="34" t="inlineStr">
-        <is>
-          <t># Placeholder for actual module integration with mesh/network.</t>
-        </is>
-      </c>
-      <c r="F5" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1" s="25">
-      <c r="A6" s="35" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="35" t="inlineStr">
-        <is>
-          <t>research_module.py</t>
-        </is>
-      </c>
-      <c r="C6" s="35" t="inlineStr">
-        <is>
-          <t>315</t>
-        </is>
-      </c>
-      <c r="D6" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E6" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F6" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="25">
-      <c r="A7" s="35" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="35" t="inlineStr">
-        <is>
-          <t>tenant_defense.py</t>
-        </is>
-      </c>
-      <c r="C7" s="35" t="inlineStr">
-        <is>
-          <t>1284</t>
-        </is>
-      </c>
-      <c r="D7" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E7" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F7" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="25">
-      <c r="A8" s="33" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="33" t="inlineStr">
-        <is>
-          <t>admin_console\module_flags.py</t>
-        </is>
-      </c>
-      <c r="C8" s="33" t="inlineStr">
-        <is>
-          <t>334</t>
-        </is>
-      </c>
-      <c r="D8" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E8" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F8" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="25">
-      <c r="A9" s="33" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="33" t="inlineStr">
-        <is>
-          <t>admin_console\router.py</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="inlineStr">
-        <is>
-          <t>1812</t>
-        </is>
-      </c>
-      <c r="D9" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E9" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F9" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="25">
-      <c r="A10" s="33" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="33" t="inlineStr">
-        <is>
-          <t>advocate\router.py</t>
-        </is>
-      </c>
-      <c r="C10" s="33" t="inlineStr">
-        <is>
-          <t>142</t>
-        </is>
-      </c>
-      <c r="D10" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E10" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F10" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="25">
-      <c r="A11" s="33" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="33" t="inlineStr">
-        <is>
-          <t>analytics\router.py</t>
-        </is>
-      </c>
-      <c r="C11" s="33" t="inlineStr">
-        <is>
-          <t>323</t>
-        </is>
-      </c>
-      <c r="D11" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E11" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F11" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="25">
-      <c r="A12" s="33" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="33" t="inlineStr">
-        <is>
-          <t>brain\router.py</t>
-        </is>
-      </c>
-      <c r="C12" s="33" t="inlineStr">
-        <is>
-          <t>321</t>
-        </is>
-      </c>
-      <c r="D12" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E12" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F12" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="25">
-      <c r="A13" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="33" t="inlineStr">
-        <is>
-          <t>case_builder\router.py</t>
-        </is>
-      </c>
-      <c r="C13" s="33" t="inlineStr">
-        <is>
-          <t>923</t>
-        </is>
-      </c>
-      <c r="D13" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E13" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F13" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="15" customHeight="1" s="25">
-      <c r="A14" s="35" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="35" t="inlineStr">
-        <is>
-          <t>case_builder\router.py</t>
-        </is>
-      </c>
-      <c r="C14" s="35" t="inlineStr">
-        <is>
-          <t>1022</t>
-        </is>
-      </c>
-      <c r="D14" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E14" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F14" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="25">
-      <c r="A15" s="34" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="34" t="inlineStr">
-        <is>
-          <t>case_builder\router.py</t>
-        </is>
-      </c>
-      <c r="C15" s="34" t="inlineStr">
-        <is>
-          <t>1930</t>
-        </is>
-      </c>
-      <c r="D15" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E15" s="34" t="inlineStr">
-        <is>
-          <t>for placeholder, value in replacements.items():</t>
-        </is>
-      </c>
-      <c r="F15" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="15" customHeight="1" s="25">
-      <c r="A16" s="34" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="34" t="inlineStr">
-        <is>
-          <t>case_builder\router.py</t>
-        </is>
-      </c>
-      <c r="C16" s="34" t="inlineStr">
-        <is>
-          <t>1931</t>
-        </is>
-      </c>
-      <c r="D16" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E16" s="34" t="inlineStr">
-        <is>
-          <t>doc_text = doc_text.replace(placeholder, value)</t>
-        </is>
-      </c>
-      <c r="F16" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="25">
-      <c r="A17" s="33" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="33" t="inlineStr">
-        <is>
-          <t>case_builder\router.py</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="inlineStr">
-        <is>
-          <t>1971</t>
-        </is>
-      </c>
-      <c r="D17" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E17" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F17" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="15" customHeight="1" s="25">
-      <c r="A18" s="33" t="n">
-        <v>17</v>
-      </c>
-      <c r="B18" s="33" t="inlineStr">
-        <is>
-          <t>case_builder\router.py</t>
-        </is>
-      </c>
-      <c r="C18" s="33" t="inlineStr">
-        <is>
-          <t>1986</t>
-        </is>
-      </c>
-      <c r="D18" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E18" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F18" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="15" customHeight="1" s="25">
-      <c r="A19" s="33" t="n">
-        <v>18</v>
-      </c>
-      <c r="B19" s="33" t="inlineStr">
-        <is>
-          <t>cloud_sync\router.py</t>
-        </is>
-      </c>
-      <c r="C19" s="33" t="inlineStr">
-        <is>
-          <t>520</t>
-        </is>
-      </c>
-      <c r="D19" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E19" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F19" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="15" customHeight="1" s="25">
-      <c r="A20" s="35" t="n">
-        <v>19</v>
-      </c>
-      <c r="B20" s="35" t="inlineStr">
-        <is>
-          <t>cloud_sync\service.py</t>
-        </is>
-      </c>
-      <c r="C20" s="35" t="inlineStr">
-        <is>
-          <t>298</t>
-        </is>
-      </c>
-      <c r="D20" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E20" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F20" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="15" customHeight="1" s="25">
-      <c r="A21" s="35" t="n">
-        <v>20</v>
-      </c>
-      <c r="B21" s="35" t="inlineStr">
-        <is>
-          <t>cloud_sync\service.py</t>
-        </is>
-      </c>
-      <c r="C21" s="35" t="inlineStr">
-        <is>
-          <t>335</t>
-        </is>
-      </c>
-      <c r="D21" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E21" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F21" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="15" customHeight="1" s="25">
-      <c r="A22" s="35" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="35" t="inlineStr">
-        <is>
-          <t>cloud_sync\service.py</t>
-        </is>
-      </c>
-      <c r="C22" s="35" t="inlineStr">
-        <is>
-          <t>366</t>
-        </is>
-      </c>
-      <c r="D22" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E22" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F22" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="15" customHeight="1" s="25">
-      <c r="A23" s="34" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="34" t="inlineStr">
-        <is>
-          <t>communication\router.py</t>
-        </is>
-      </c>
-      <c r="C23" s="34" t="inlineStr">
-        <is>
-          <t>486</t>
-        </is>
-      </c>
-      <c r="D23" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E23" s="34" t="inlineStr">
-        <is>
-          <t># WebSocket / Real-time (Placeholder)</t>
-        </is>
-      </c>
-      <c r="F23" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="15" customHeight="1" s="25">
-      <c r="A24" s="34" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="34" t="inlineStr">
-        <is>
-          <t>communication\router.py</t>
-        </is>
-      </c>
-      <c r="C24" s="34" t="inlineStr">
-        <is>
-          <t>501</t>
-        </is>
-      </c>
-      <c r="D24" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E24" s="34" t="inlineStr">
-        <is>
-          <t>This is a placeholder for real-time typing indicators.</t>
-        </is>
-      </c>
-      <c r="F24" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="15" customHeight="1" s="25">
-      <c r="A25" s="34" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="34" t="inlineStr">
-        <is>
-          <t>communication\service.py</t>
-        </is>
-      </c>
-      <c r="C25" s="34" t="inlineStr">
-        <is>
-          <t>83</t>
-        </is>
-      </c>
-      <c r="D25" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E25" s="34" t="inlineStr">
-        <is>
-          <t>name=recipient_id  # Placeholder</t>
-        </is>
-      </c>
-      <c r="F25" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="15" customHeight="1" s="25">
-      <c r="A26" s="35" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="35" t="inlineStr">
-        <is>
-          <t>communication\service.py</t>
-        </is>
-      </c>
-      <c r="C26" s="35" t="inlineStr">
-        <is>
-          <t>558</t>
-        </is>
-      </c>
-      <c r="D26" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E26" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F26" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="15" customHeight="1" s="25">
-      <c r="A27" s="33" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="33" t="inlineStr">
-        <is>
-          <t>components\router.py</t>
-        </is>
-      </c>
-      <c r="C27" s="33" t="inlineStr">
-        <is>
-          <t>271</t>
-        </is>
-      </c>
-      <c r="D27" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E27" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F27" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="15" customHeight="1" s="25">
-      <c r="A28" s="33" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="33" t="inlineStr">
-        <is>
-          <t>components\router.py</t>
-        </is>
-      </c>
-      <c r="C28" s="33" t="inlineStr">
-        <is>
-          <t>315</t>
-        </is>
-      </c>
-      <c r="D28" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E28" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F28" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="15" customHeight="1" s="25">
-      <c r="A29" s="33" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="33" t="inlineStr">
-        <is>
-          <t>components\router.py</t>
-        </is>
-      </c>
-      <c r="C29" s="33" t="inlineStr">
-        <is>
-          <t>354</t>
-        </is>
-      </c>
-      <c r="D29" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E29" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F29" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="15" customHeight="1" s="25">
-      <c r="A30" s="33" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="33" t="inlineStr">
-        <is>
-          <t>components\router.py</t>
-        </is>
-      </c>
-      <c r="C30" s="33" t="inlineStr">
-        <is>
-          <t>386</t>
-        </is>
-      </c>
-      <c r="D30" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E30" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F30" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="15" customHeight="1" s="25">
-      <c r="A31" s="33" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="33" t="inlineStr">
-        <is>
-          <t>components\router.py</t>
-        </is>
-      </c>
-      <c r="C31" s="33" t="inlineStr">
-        <is>
-          <t>422</t>
-        </is>
-      </c>
-      <c r="D31" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E31" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F31" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="15" customHeight="1" s="25">
-      <c r="A32" s="33" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="33" t="inlineStr">
-        <is>
-          <t>components\router.py</t>
-        </is>
-      </c>
-      <c r="C32" s="33" t="inlineStr">
-        <is>
-          <t>493</t>
-        </is>
-      </c>
-      <c r="D32" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E32" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F32" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="15" customHeight="1" s="25">
-      <c r="A33" s="33" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="33" t="inlineStr">
-        <is>
-          <t>components\router.py</t>
-        </is>
-      </c>
-      <c r="C33" s="33" t="inlineStr">
-        <is>
-          <t>531</t>
-        </is>
-      </c>
-      <c r="D33" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E33" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F33" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="15" customHeight="1" s="25">
-      <c r="A34" s="33" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="33" t="inlineStr">
-        <is>
-          <t>components\router.py</t>
-        </is>
-      </c>
-      <c r="C34" s="33" t="inlineStr">
-        <is>
-          <t>604</t>
-        </is>
-      </c>
-      <c r="D34" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E34" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F34" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="15" customHeight="1" s="25">
-      <c r="A35" s="33" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="33" t="inlineStr">
-        <is>
-          <t>components\router.py</t>
-        </is>
-      </c>
-      <c r="C35" s="33" t="inlineStr">
-        <is>
-          <t>697</t>
-        </is>
-      </c>
-      <c r="D35" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E35" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F35" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="15" customHeight="1" s="25">
-      <c r="A36" s="33" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="33" t="inlineStr">
-        <is>
-          <t>components\router.py</t>
-        </is>
-      </c>
-      <c r="C36" s="33" t="inlineStr">
-        <is>
-          <t>708</t>
-        </is>
-      </c>
-      <c r="D36" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E36" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F36" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="15" customHeight="1" s="25">
-      <c r="A37" s="33" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="33" t="inlineStr">
-        <is>
-          <t>components\router.py</t>
-        </is>
-      </c>
-      <c r="C37" s="33" t="inlineStr">
-        <is>
-          <t>756</t>
-        </is>
-      </c>
-      <c r="D37" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E37" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F37" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="15" customHeight="1" s="25">
-      <c r="A38" s="35" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="35" t="inlineStr">
-        <is>
-          <t>context_engine\gatherer.py</t>
-        </is>
-      </c>
-      <c r="C38" s="35" t="inlineStr">
-        <is>
-          <t>52</t>
-        </is>
-      </c>
-      <c r="D38" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E38" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F38" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="15" customHeight="1" s="25">
-      <c r="A39" s="35" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="35" t="inlineStr">
-        <is>
-          <t>context_engine\gatherer.py</t>
-        </is>
-      </c>
-      <c r="C39" s="35" t="inlineStr">
-        <is>
-          <t>58</t>
-        </is>
-      </c>
-      <c r="D39" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E39" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F39" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="15" customHeight="1" s="25">
-      <c r="A40" s="33" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="33" t="inlineStr">
-        <is>
-          <t>court_forms\router.py</t>
-        </is>
-      </c>
-      <c r="C40" s="33" t="inlineStr">
-        <is>
-          <t>436</t>
-        </is>
-      </c>
-      <c r="D40" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E40" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F40" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="15" customHeight="1" s="25">
-      <c r="A41" s="33" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="33" t="inlineStr">
-        <is>
-          <t>court_forms\router.py</t>
-        </is>
-      </c>
-      <c r="C41" s="33" t="inlineStr">
-        <is>
-          <t>449</t>
-        </is>
-      </c>
-      <c r="D41" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E41" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F41" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="15" customHeight="1" s="25">
-      <c r="A42" s="33" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="33" t="inlineStr">
-        <is>
-          <t>court_forms\router.py</t>
-        </is>
-      </c>
-      <c r="C42" s="33" t="inlineStr">
-        <is>
-          <t>516</t>
-        </is>
-      </c>
-      <c r="D42" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E42" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F42" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="15" customHeight="1" s="25">
-      <c r="A43" s="33" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" s="33" t="inlineStr">
-        <is>
-          <t>court_forms\router.py</t>
-        </is>
-      </c>
-      <c r="C43" s="33" t="inlineStr">
-        <is>
-          <t>529</t>
-        </is>
-      </c>
-      <c r="D43" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E43" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F43" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="15" customHeight="1" s="25">
-      <c r="A44" s="33" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="33" t="inlineStr">
-        <is>
-          <t>court_forms\router.py</t>
-        </is>
-      </c>
-      <c r="C44" s="33" t="inlineStr">
-        <is>
-          <t>798</t>
-        </is>
-      </c>
-      <c r="D44" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E44" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F44" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="15" customHeight="1" s="25">
-      <c r="A45" s="33" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" s="33" t="inlineStr">
-        <is>
-          <t>court_forms\service.py</t>
-        </is>
-      </c>
-      <c r="C45" s="33" t="inlineStr">
-        <is>
-          <t>565</t>
-        </is>
-      </c>
-      <c r="D45" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E45" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F45" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="15" customHeight="1" s="25">
-      <c r="A46" s="33" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="33" t="inlineStr">
-        <is>
-          <t>court_forms\service.py</t>
-        </is>
-      </c>
-      <c r="C46" s="33" t="inlineStr">
-        <is>
-          <t>573</t>
-        </is>
-      </c>
-      <c r="D46" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E46" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F46" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="15" customHeight="1" s="25">
-      <c r="A47" s="35" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="35" t="inlineStr">
-        <is>
-          <t>court_packet\router.py</t>
-        </is>
-      </c>
-      <c r="C47" s="35" t="inlineStr">
-        <is>
-          <t>49</t>
-        </is>
-      </c>
-      <c r="D47" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E47" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F47" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="15" customHeight="1" s="25">
-      <c r="A48" s="34" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="34" t="inlineStr">
-        <is>
-          <t>court_packet\router.py</t>
-        </is>
-      </c>
-      <c r="C48" s="34" t="inlineStr">
-        <is>
-          <t>361</t>
-        </is>
-      </c>
-      <c r="D48" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E48" s="34" t="inlineStr">
-        <is>
-          <t># For now, create placeholder with metadata</t>
-        </is>
-      </c>
-      <c r="F48" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="15" customHeight="1" s="25">
-      <c r="A49" s="33" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" s="33" t="inlineStr">
-        <is>
-          <t>crawler\service.py</t>
-        </is>
-      </c>
-      <c r="C49" s="33" t="inlineStr">
-        <is>
-          <t>292</t>
-        </is>
-      </c>
-      <c r="D49" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E49" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F49" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="15" customHeight="1" s="25">
-      <c r="A50" s="35" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="35" t="inlineStr">
-        <is>
-          <t>crawler\service.py</t>
-        </is>
-      </c>
-      <c r="C50" s="35" t="inlineStr">
-        <is>
-          <t>590</t>
-        </is>
-      </c>
-      <c r="D50" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E50" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F50" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="15" customHeight="1" s="25">
-      <c r="A51" s="34" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" s="34" t="inlineStr">
-        <is>
-          <t>development\router.py</t>
-        </is>
-      </c>
-      <c r="C51" s="34" t="inlineStr">
-        <is>
-          <t>243</t>
-        </is>
-      </c>
-      <c r="D51" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E51" s="34" t="inlineStr">
-        <is>
-          <t># Placeholder for different analysis types</t>
-        </is>
-      </c>
-      <c r="F51" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="15" customHeight="1" s="25">
-      <c r="A52" s="33" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" s="33" t="inlineStr">
-        <is>
-          <t>dev_lab\ideas.py</t>
-        </is>
-      </c>
-      <c r="C52" s="33" t="inlineStr">
-        <is>
-          <t>382</t>
-        </is>
-      </c>
-      <c r="D52" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E52" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F52" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="15" customHeight="1" s="25">
-      <c r="A53" s="33" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" s="33" t="inlineStr">
-        <is>
-          <t>dev_lab\maturity.py</t>
-        </is>
-      </c>
-      <c r="C53" s="33" t="inlineStr">
-        <is>
-          <t>42</t>
-        </is>
-      </c>
-      <c r="D53" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E53" s="33" t="inlineStr">
-        <is>
-          <t>"No dev_notes or TODO markers for core functionality",</t>
-        </is>
-      </c>
-      <c r="F53" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="15" customHeight="1" s="25">
-      <c r="A54" s="33" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" s="33" t="inlineStr">
-        <is>
-          <t>dev_lab\maturity.py</t>
-        </is>
-      </c>
-      <c r="C54" s="33" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="D54" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E54" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F54" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="15" customHeight="1" s="25">
-      <c r="A55" s="33" t="n">
-        <v>54</v>
-      </c>
-      <c r="B55" s="33" t="inlineStr">
-        <is>
-          <t>dev_lab\router.py</t>
-        </is>
-      </c>
-      <c r="C55" s="33" t="inlineStr">
-        <is>
-          <t>331</t>
-        </is>
-      </c>
-      <c r="D55" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E55" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F55" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="15" customHeight="1" s="25">
-      <c r="A56" s="33" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" s="33" t="inlineStr">
-        <is>
-          <t>dev_lab\router.py</t>
-        </is>
-      </c>
-      <c r="C56" s="33" t="inlineStr">
-        <is>
-          <t>426</t>
-        </is>
-      </c>
-      <c r="D56" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E56" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F56" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="15" customHeight="1" s="25">
-      <c r="A57" s="35" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" s="35" t="inlineStr">
-        <is>
-          <t>documents\router.py</t>
-        </is>
-      </c>
-      <c r="C57" s="35" t="inlineStr">
-        <is>
-          <t>161</t>
-        </is>
-      </c>
-      <c r="D57" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E57" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F57" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="15" customHeight="1" s="25">
-      <c r="A58" s="35" t="n">
-        <v>57</v>
-      </c>
-      <c r="B58" s="35" t="inlineStr">
-        <is>
-          <t>document_center\router.py</t>
-        </is>
-      </c>
-      <c r="C58" s="35" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="D58" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E58" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F58" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="15" customHeight="1" s="25">
-      <c r="A59" s="35" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" s="35" t="inlineStr">
-        <is>
-          <t>document_center\router.py</t>
-        </is>
-      </c>
-      <c r="C59" s="35" t="inlineStr">
-        <is>
-          <t>82</t>
-        </is>
-      </c>
-      <c r="D59" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E59" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F59" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="15" customHeight="1" s="25">
-      <c r="A60" s="35" t="n">
-        <v>59</v>
-      </c>
-      <c r="B60" s="35" t="inlineStr">
-        <is>
-          <t>document_center\router.py</t>
-        </is>
-      </c>
-      <c r="C60" s="35" t="inlineStr">
-        <is>
-          <t>85</t>
-        </is>
-      </c>
-      <c r="D60" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E60" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F60" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="15" customHeight="1" s="25">
-      <c r="A61" s="34" t="n">
-        <v>60</v>
-      </c>
-      <c r="B61" s="34" t="inlineStr">
-        <is>
-          <t>document_delivery\router.py</t>
-        </is>
-      </c>
-      <c r="C61" s="34" t="inlineStr">
-        <is>
-          <t>146</t>
-        </is>
-      </c>
-      <c r="D61" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E61" s="34" t="inlineStr">
-        <is>
-          <t>document_hash = "placeholder_hash"  # Would compute from actual document</t>
-        </is>
-      </c>
-      <c r="F61" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="15" customHeight="1" s="25">
-      <c r="A62" s="34" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" s="34" t="inlineStr">
-        <is>
-          <t>emotion\router.py</t>
-        </is>
-      </c>
-      <c r="C62" s="34" t="inlineStr">
-        <is>
-          <t>160</t>
-        </is>
-      </c>
-      <c r="D62" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E62" s="34" t="inlineStr">
-        <is>
-          <t>{"name": "deadline_approaching", "description": "Deadline coming soon"},</t>
-        </is>
-      </c>
-      <c r="F62" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="15" customHeight="1" s="25">
-      <c r="A63" s="33" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" s="33" t="inlineStr">
-        <is>
-          <t>enterprise_dashboard\router.py</t>
-        </is>
-      </c>
-      <c r="C63" s="33" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="D63" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E63" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F63" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" ht="15" customHeight="1" s="25">
-      <c r="A64" s="33" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" s="33" t="inlineStr">
-        <is>
-          <t>extraction\service.py</t>
-        </is>
-      </c>
-      <c r="C64" s="33" t="inlineStr">
-        <is>
-          <t>805</t>
-        </is>
-      </c>
-      <c r="D64" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E64" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F64" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="15" customHeight="1" s="25">
-      <c r="A65" s="34" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" s="34" t="inlineStr">
-        <is>
-          <t>filedored\gui_requirements.py</t>
-        </is>
-      </c>
-      <c r="C65" s="34" t="inlineStr">
-        <is>
-          <t>34</t>
-        </is>
-      </c>
-      <c r="D65" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E65" s="34" t="inlineStr">
-        <is>
-          <t>placeholder="Search by filename or content...",</t>
-        </is>
-      </c>
-      <c r="F65" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="66" ht="15" customHeight="1" s="25">
-      <c r="A66" s="33" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" s="33" t="inlineStr">
-        <is>
-          <t>form_data\router.py</t>
-        </is>
-      </c>
-      <c r="C66" s="33" t="inlineStr">
-        <is>
-          <t>177</t>
-        </is>
-      </c>
-      <c r="D66" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E66" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F66" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="15" customHeight="1" s="25">
-      <c r="A67" s="33" t="n">
-        <v>66</v>
-      </c>
-      <c r="B67" s="33" t="inlineStr">
-        <is>
-          <t>form_data\router.py</t>
-        </is>
-      </c>
-      <c r="C67" s="33" t="inlineStr">
-        <is>
-          <t>242</t>
-        </is>
-      </c>
-      <c r="D67" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E67" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F67" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="15" customHeight="1" s="25">
-      <c r="A68" s="33" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" s="33" t="inlineStr">
-        <is>
-          <t>funding_mgmt\schemas.py</t>
-        </is>
-      </c>
-      <c r="C68" s="33" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="D68" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E68" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F68" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="15" customHeight="1" s="25">
-      <c r="A69" s="33" t="n">
-        <v>68</v>
-      </c>
-      <c r="B69" s="33" t="inlineStr">
-        <is>
-          <t>funding_mgmt\schemas.py</t>
-        </is>
-      </c>
-      <c r="C69" s="33" t="inlineStr">
-        <is>
-          <t>89</t>
-        </is>
-      </c>
-      <c r="D69" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E69" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F69" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="15" customHeight="1" s="25">
-      <c r="A70" s="33" t="n">
-        <v>69</v>
-      </c>
-      <c r="B70" s="33" t="inlineStr">
-        <is>
-          <t>health\router.py</t>
-        </is>
-      </c>
-      <c r="C70" s="33" t="inlineStr">
-        <is>
-          <t>95</t>
-        </is>
-      </c>
-      <c r="D70" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E70" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F70" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="71" ht="15" customHeight="1" s="25">
-      <c r="A71" s="33" t="n">
-        <v>70</v>
-      </c>
-      <c r="B71" s="33" t="inlineStr">
-        <is>
-          <t>housing_accountability\router.py</t>
-        </is>
-      </c>
-      <c r="C71" s="33" t="inlineStr">
-        <is>
-          <t>535</t>
-        </is>
-      </c>
-      <c r="D71" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E71" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F71" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="15" customHeight="1" s="25">
-      <c r="A72" s="35" t="n">
-        <v>71</v>
-      </c>
-      <c r="B72" s="35" t="inlineStr">
-        <is>
-          <t>housing_accountability\router.py</t>
-        </is>
-      </c>
-      <c r="C72" s="35" t="inlineStr">
-        <is>
-          <t>948</t>
-        </is>
-      </c>
-      <c r="D72" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E72" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F72" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" ht="15" customHeight="1" s="25">
-      <c r="A73" s="35" t="n">
-        <v>72</v>
-      </c>
-      <c r="B73" s="35" t="inlineStr">
-        <is>
-          <t>hud_funding\service.py</t>
-        </is>
-      </c>
-      <c r="C73" s="35" t="inlineStr">
-        <is>
-          <t>1274</t>
-        </is>
-      </c>
-      <c r="D73" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E73" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F73" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="74" ht="15" customHeight="1" s="25">
-      <c r="A74" s="35" t="n">
-        <v>73</v>
-      </c>
-      <c r="B74" s="35" t="inlineStr">
-        <is>
-          <t>hud_funding\service.py</t>
-        </is>
-      </c>
-      <c r="C74" s="35" t="inlineStr">
-        <is>
-          <t>1300</t>
-        </is>
-      </c>
-      <c r="D74" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E74" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F74" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="75" ht="15" customHeight="1" s="25">
-      <c r="A75" s="35" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" s="35" t="inlineStr">
-        <is>
-          <t>intake\router.py</t>
-        </is>
-      </c>
-      <c r="C75" s="35" t="inlineStr">
-        <is>
-          <t>87</t>
-        </is>
-      </c>
-      <c r="D75" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E75" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F75" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="76" ht="15" customHeight="1" s="25">
-      <c r="A76" s="34" t="n">
-        <v>75</v>
-      </c>
-      <c r="B76" s="34" t="inlineStr">
-        <is>
-          <t>intake\router.py</t>
-        </is>
-      </c>
-      <c r="C76" s="34" t="inlineStr">
-        <is>
-          <t>451</t>
-        </is>
-      </c>
-      <c r="D76" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E76" s="34" t="inlineStr">
-        <is>
-          <t># Resolve storage provider from user if not provided or placeholder</t>
-        </is>
-      </c>
-      <c r="F76" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="15" customHeight="1" s="25">
-      <c r="A77" s="33" t="n">
-        <v>76</v>
-      </c>
-      <c r="B77" s="33" t="inlineStr">
-        <is>
-          <t>intake\router.py</t>
-        </is>
-      </c>
-      <c r="C77" s="33" t="inlineStr">
-        <is>
-          <t>517</t>
-        </is>
-      </c>
-      <c r="D77" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E77" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F77" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="15" customHeight="1" s="25">
-      <c r="A78" s="33" t="n">
-        <v>77</v>
-      </c>
-      <c r="B78" s="33" t="inlineStr">
-        <is>
-          <t>intake\router.py</t>
-        </is>
-      </c>
-      <c r="C78" s="33" t="inlineStr">
-        <is>
-          <t>805</t>
-        </is>
-      </c>
-      <c r="D78" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E78" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F78" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" ht="15" customHeight="1" s="25">
-      <c r="A79" s="33" t="n">
-        <v>78</v>
-      </c>
-      <c r="B79" s="33" t="inlineStr">
-        <is>
-          <t>intake\router.py</t>
-        </is>
-      </c>
-      <c r="C79" s="33" t="inlineStr">
-        <is>
-          <t>945</t>
-        </is>
-      </c>
-      <c r="D79" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E79" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F79" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="15" customHeight="1" s="25">
-      <c r="A80" s="35" t="n">
-        <v>79</v>
-      </c>
-      <c r="B80" s="35" t="inlineStr">
-        <is>
-          <t>intake\service.py</t>
-        </is>
-      </c>
-      <c r="C80" s="35" t="inlineStr">
-        <is>
-          <t>358</t>
-        </is>
-      </c>
-      <c r="D80" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E80" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F80" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" ht="15" customHeight="1" s="25">
-      <c r="A81" s="34" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" s="34" t="inlineStr">
-        <is>
-          <t>law_library\router.py</t>
-        </is>
-      </c>
-      <c r="C81" s="34" t="inlineStr">
-        <is>
-          <t>2365</t>
-        </is>
-      </c>
-      <c r="D81" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E81" s="34" t="inlineStr">
-        <is>
-          <t>.search-box input::placeholder { color: #a7f3d0; }</t>
-        </is>
-      </c>
-      <c r="F81" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="82" ht="15" customHeight="1" s="25">
-      <c r="A82" s="34" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" s="34" t="inlineStr">
-        <is>
-          <t>law_library\router.py</t>
-        </is>
-      </c>
-      <c r="C82" s="34" t="inlineStr">
-        <is>
-          <t>2396</t>
-        </is>
-      </c>
-      <c r="D82" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E82" s="34" t="inlineStr">
-        <is>
-          <t>&lt;input type="text" id="search-input" placeholder="Search statutes, case law, rig</t>
-        </is>
-      </c>
-      <c r="F82" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="15" customHeight="1" s="25">
-      <c r="A83" s="34" t="n">
-        <v>82</v>
-      </c>
-      <c r="B83" s="34" t="inlineStr">
-        <is>
-          <t>law_library\router.py</t>
-        </is>
-      </c>
-      <c r="C83" s="34" t="inlineStr">
-        <is>
-          <t>2414</t>
-        </is>
-      </c>
-      <c r="D83" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E83" s="34" t="inlineStr">
-        <is>
-          <t>&lt;input type="text" id="chat-input" placeholder="Ask about tenant rights, evictio</t>
-        </is>
-      </c>
-      <c r="F83" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="15" customHeight="1" s="25">
-      <c r="A84" s="35" t="n">
-        <v>83</v>
-      </c>
-      <c r="B84" s="35" t="inlineStr">
-        <is>
-          <t>legal_filing\service.py</t>
-        </is>
-      </c>
-      <c r="C84" s="35" t="inlineStr">
-        <is>
-          <t>63</t>
-        </is>
-      </c>
-      <c r="D84" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E84" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F84" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="15" customHeight="1" s="25">
-      <c r="A85" s="35" t="n">
-        <v>84</v>
-      </c>
-      <c r="B85" s="35" t="inlineStr">
-        <is>
-          <t>legal_filing\service.py</t>
-        </is>
-      </c>
-      <c r="C85" s="35" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
-      </c>
-      <c r="D85" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E85" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F85" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="86" ht="15" customHeight="1" s="25">
-      <c r="A86" s="35" t="n">
-        <v>85</v>
-      </c>
-      <c r="B86" s="35" t="inlineStr">
-        <is>
-          <t>legal_filing\service.py</t>
-        </is>
-      </c>
-      <c r="C86" s="35" t="inlineStr">
-        <is>
-          <t>71</t>
-        </is>
-      </c>
-      <c r="D86" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E86" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F86" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="15" customHeight="1" s="25">
-      <c r="A87" s="35" t="n">
-        <v>86</v>
-      </c>
-      <c r="B87" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\court_scraper.py</t>
-        </is>
-      </c>
-      <c r="C87" s="35" t="inlineStr">
-        <is>
-          <t>68</t>
-        </is>
-      </c>
-      <c r="D87" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E87" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F87" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="15" customHeight="1" s="25">
-      <c r="A88" s="35" t="n">
-        <v>87</v>
-      </c>
-      <c r="B88" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\court_scraper.py</t>
-        </is>
-      </c>
-      <c r="C88" s="35" t="inlineStr">
-        <is>
-          <t>115</t>
-        </is>
-      </c>
-      <c r="D88" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E88" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F88" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="15" customHeight="1" s="25">
-      <c r="A89" s="35" t="n">
-        <v>88</v>
-      </c>
-      <c r="B89" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\court_scraper.py</t>
-        </is>
-      </c>
-      <c r="C89" s="35" t="inlineStr">
-        <is>
-          <t>158</t>
-        </is>
-      </c>
-      <c r="D89" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E89" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F89" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="15" customHeight="1" s="25">
-      <c r="A90" s="35" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\gui_butler.py</t>
-        </is>
-      </c>
-      <c r="C90" s="35" t="inlineStr">
-        <is>
-          <t>358</t>
-        </is>
-      </c>
-      <c r="D90" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E90" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F90" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="15" customHeight="1" s="25">
-      <c r="A91" s="35" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\gui_butler.py</t>
-        </is>
-      </c>
-      <c r="C91" s="35" t="inlineStr">
-        <is>
-          <t>386</t>
-        </is>
-      </c>
-      <c r="D91" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E91" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F91" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="15" customHeight="1" s="25">
-      <c r="A92" s="35" t="n">
-        <v>91</v>
-      </c>
-      <c r="B92" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\gui_butler.py</t>
-        </is>
-      </c>
-      <c r="C92" s="35" t="inlineStr">
-        <is>
-          <t>407</t>
-        </is>
-      </c>
-      <c r="D92" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E92" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F92" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="93" ht="15" customHeight="1" s="25">
-      <c r="A93" s="35" t="n">
-        <v>92</v>
-      </c>
-      <c r="B93" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\gui_butler.py</t>
-        </is>
-      </c>
-      <c r="C93" s="35" t="inlineStr">
-        <is>
-          <t>444</t>
-        </is>
-      </c>
-      <c r="D93" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E93" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F93" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="15" customHeight="1" s="25">
-      <c r="A94" s="35" t="n">
-        <v>93</v>
-      </c>
-      <c r="B94" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\gui_butler.py</t>
-        </is>
-      </c>
-      <c r="C94" s="35" t="inlineStr">
-        <is>
-          <t>465</t>
-        </is>
-      </c>
-      <c r="D94" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E94" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F94" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="15" customHeight="1" s="25">
-      <c r="A95" s="35" t="n">
-        <v>94</v>
-      </c>
-      <c r="B95" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\gui_butler.py</t>
-        </is>
-      </c>
-      <c r="C95" s="35" t="inlineStr">
-        <is>
-          <t>494</t>
-        </is>
-      </c>
-      <c r="D95" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E95" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F95" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="15" customHeight="1" s="25">
-      <c r="A96" s="34" t="n">
-        <v>95</v>
-      </c>
-      <c r="B96" s="34" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\intelligence_engine.py</t>
-        </is>
-      </c>
-      <c r="C96" s="34" t="inlineStr">
-        <is>
-          <t>524</t>
-        </is>
-      </c>
-      <c r="D96" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E96" s="34" t="inlineStr">
-        <is>
-          <t># For now, return a placeholder</t>
-        </is>
-      </c>
-      <c r="F96" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="15" customHeight="1" s="25">
-      <c r="A97" s="34" t="n">
-        <v>96</v>
-      </c>
-      <c r="B97" s="34" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\reporting_layer.py</t>
-        </is>
-      </c>
-      <c r="C97" s="34" t="inlineStr">
-        <is>
-          <t>404</t>
-        </is>
-      </c>
-      <c r="D97" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E97" s="34" t="inlineStr">
-        <is>
-          <t># For now, return a placeholder</t>
-        </is>
-      </c>
-      <c r="F97" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="15" customHeight="1" s="25">
-      <c r="A98" s="34" t="n">
-        <v>97</v>
-      </c>
-      <c r="B98" s="34" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\reporting_layer.py</t>
-        </is>
-      </c>
-      <c r="C98" s="34" t="inlineStr">
-        <is>
-          <t>414</t>
-        </is>
-      </c>
-      <c r="D98" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E98" s="34" t="inlineStr">
-        <is>
-          <t># For now, return placeholder metrics</t>
-        </is>
-      </c>
-      <c r="F98" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" ht="23.25" customHeight="1" s="25">
-      <c r="A99" s="33" t="n">
-        <v>98</v>
-      </c>
-      <c r="B99" s="33" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\router.py</t>
-        </is>
-      </c>
-      <c r="C99" s="33" t="inlineStr">
-        <is>
-          <t>21</t>
-        </is>
-      </c>
-      <c r="D99" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E99" s="33" t="inlineStr">
-        <is>
-          <t># from .graph_engine import create_graph_engine  # TODO: graph_engine not implem</t>
-        </is>
-      </c>
-      <c r="F99" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="23.25" customHeight="1" s="25">
-      <c r="A100" s="33" t="n">
-        <v>99</v>
-      </c>
-      <c r="B100" s="33" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\router.py</t>
-        </is>
-      </c>
-      <c r="C100" s="33" t="inlineStr">
-        <is>
-          <t>81</t>
-        </is>
-      </c>
-      <c r="D100" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E100" s="33" t="inlineStr">
-        <is>
-          <t># graph_engine = create_graph_engine()  # TODO: graph_engine not implemented</t>
-        </is>
-      </c>
-      <c r="F100" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="23.25" customHeight="1" s="25">
-      <c r="A101" s="33" t="n">
-        <v>100</v>
-      </c>
-      <c r="B101" s="33" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\router.py</t>
-        </is>
-      </c>
-      <c r="C101" s="33" t="inlineStr">
-        <is>
-          <t>452</t>
-        </is>
-      </c>
-      <c r="D101" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E101" s="33" t="inlineStr">
-        <is>
-          <t># graph_stats = graph_engine.analyze_graph()  # TODO: graph_engine not implement</t>
-        </is>
-      </c>
-      <c r="F101" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="23.25" customHeight="1" s="25">
-      <c r="A102" s="33" t="n">
-        <v>101</v>
-      </c>
-      <c r="B102" s="33" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\router.py</t>
-        </is>
-      </c>
-      <c r="C102" s="33" t="inlineStr">
-        <is>
-          <t>460</t>
-        </is>
-      </c>
-      <c r="D102" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E102" s="33" t="inlineStr">
-        <is>
-          <t>"graph": {"status": "not_implemented"},  # TODO: graph_engine not implemented</t>
-        </is>
-      </c>
-      <c r="F102" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="15" customHeight="1" s="25">
-      <c r="A103" s="34" t="n">
-        <v>102</v>
-      </c>
-      <c r="B103" s="34" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\scheduler.py</t>
-        </is>
-      </c>
-      <c r="C103" s="34" t="inlineStr">
-        <is>
-          <t>251</t>
-        </is>
-      </c>
-      <c r="D103" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E103" s="34" t="inlineStr">
-        <is>
-          <t>storage_health = "healthy"  # Placeholder</t>
-        </is>
-      </c>
-      <c r="F103" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="15" customHeight="1" s="25">
-      <c r="A104" s="34" t="n">
-        <v>103</v>
-      </c>
-      <c r="B104" s="34" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\scheduler.py</t>
-        </is>
-      </c>
-      <c r="C104" s="34" t="inlineStr">
-        <is>
-          <t>255</t>
-        </is>
-      </c>
-      <c r="D104" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E104" s="34" t="inlineStr">
-        <is>
-          <t>external_health = "healthy"  # Placeholder</t>
-        </is>
-      </c>
-      <c r="F104" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="15" customHeight="1" s="25">
-      <c r="A105" s="35" t="n">
-        <v>104</v>
-      </c>
-      <c r="B105" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\storage_layer.py</t>
-        </is>
-      </c>
-      <c r="C105" s="35" t="inlineStr">
-        <is>
-          <t>363</t>
-        </is>
-      </c>
-      <c r="D105" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E105" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F105" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="106" ht="15" customHeight="1" s="25">
-      <c r="A106" s="35" t="n">
-        <v>105</v>
-      </c>
-      <c r="B106" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\storage_layer.py</t>
-        </is>
-      </c>
-      <c r="C106" s="35" t="inlineStr">
-        <is>
-          <t>404</t>
-        </is>
-      </c>
-      <c r="D106" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E106" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F106" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="107" ht="15" customHeight="1" s="25">
-      <c r="A107" s="35" t="n">
-        <v>106</v>
-      </c>
-      <c r="B107" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\storage_layer.py</t>
-        </is>
-      </c>
-      <c r="C107" s="35" t="inlineStr">
-        <is>
-          <t>410</t>
-        </is>
-      </c>
-      <c r="D107" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E107" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F107" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="15" customHeight="1" s="25">
-      <c r="A108" s="35" t="n">
-        <v>107</v>
-      </c>
-      <c r="B108" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\storage_layer.py</t>
-        </is>
-      </c>
-      <c r="C108" s="35" t="inlineStr">
-        <is>
-          <t>435</t>
-        </is>
-      </c>
-      <c r="D108" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E108" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F108" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="15" customHeight="1" s="25">
-      <c r="A109" s="35" t="n">
-        <v>108</v>
-      </c>
-      <c r="B109" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\storage_layer.py</t>
-        </is>
-      </c>
-      <c r="C109" s="35" t="inlineStr">
-        <is>
-          <t>441</t>
-        </is>
-      </c>
-      <c r="D109" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E109" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F109" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="110" ht="15" customHeight="1" s="25">
-      <c r="A110" s="35" t="n">
-        <v>109</v>
-      </c>
-      <c r="B110" s="35" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\storage_layer.py</t>
-        </is>
-      </c>
-      <c r="C110" s="35" t="inlineStr">
-        <is>
-          <t>479</t>
-        </is>
-      </c>
-      <c r="D110" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E110" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F110" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="23.25" customHeight="1" s="25">
-      <c r="A111" s="33" t="n">
-        <v>110</v>
-      </c>
-      <c r="B111" s="33" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\__init__.py</t>
-        </is>
-      </c>
-      <c r="C111" s="33" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="D111" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E111" s="33" t="inlineStr">
-        <is>
-          <t># from .graph_engine import GraphEngine  # TODO: graph_engine not implemented ye</t>
-        </is>
-      </c>
-      <c r="F111" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="15" customHeight="1" s="25">
-      <c r="A112" s="33" t="n">
-        <v>111</v>
-      </c>
-      <c r="B112" s="33" t="inlineStr">
-        <is>
-          <t>litigation_intelligence\__init__.py</t>
-        </is>
-      </c>
-      <c r="C112" s="33" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="D112" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E112" s="33" t="inlineStr">
-        <is>
-          <t># 'GraphEngine',  # TODO: graph_engine not implemented yet</t>
-        </is>
-      </c>
-      <c r="F112" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="15" customHeight="1" s="25">
-      <c r="A113" s="34" t="n">
-        <v>112</v>
-      </c>
-      <c r="B113" s="34" t="inlineStr">
-        <is>
-          <t>onboarding\router.py</t>
-        </is>
-      </c>
-      <c r="C113" s="34" t="inlineStr">
-        <is>
-          <t>849</t>
-        </is>
-      </c>
-      <c r="D113" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E113" s="34" t="inlineStr">
-        <is>
-          <t>"""Render role selection page — all 5 roles, non-tenant marked Coming Soon."""</t>
-        </is>
-      </c>
-      <c r="F113" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="114" ht="15" customHeight="1" s="25">
-      <c r="A114" s="34" t="n">
-        <v>113</v>
-      </c>
-      <c r="B114" s="34" t="inlineStr">
-        <is>
-          <t>onboarding\router.py</t>
-        </is>
-      </c>
-      <c r="C114" s="34" t="inlineStr">
-        <is>
-          <t>874</t>
-        </is>
-      </c>
-      <c r="D114" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E114" s="34" t="inlineStr">
-        <is>
-          <t>&lt;div class="role-option coming-soon" title="Coming soon"&gt;</t>
-        </is>
-      </c>
-      <c r="F114" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="115" ht="23.25" customHeight="1" s="25">
-      <c r="A115" s="34" t="n">
-        <v>114</v>
-      </c>
-      <c r="B115" s="34" t="inlineStr">
-        <is>
-          <t>onboarding\router.py</t>
-        </is>
-      </c>
-      <c r="C115" s="34" t="inlineStr">
-        <is>
-          <t>877</t>
-        </is>
-      </c>
-      <c r="D115" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E115" s="34" t="inlineStr">
-        <is>
-          <t>&lt;div class="role-name"&gt;{name} &lt;span class="badge"&gt;Coming Soon&lt;/span&gt;&lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="F115" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="15" customHeight="1" s="25">
-      <c r="A116" s="33" t="n">
-        <v>115</v>
-      </c>
-      <c r="B116" s="33" t="inlineStr">
-        <is>
-          <t>page_editor\router.py</t>
-        </is>
-      </c>
-      <c r="C116" s="33" t="inlineStr">
-        <is>
-          <t>299</t>
-        </is>
-      </c>
-      <c r="D116" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E116" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F116" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="117" ht="15" customHeight="1" s="25">
-      <c r="A117" s="33" t="n">
-        <v>116</v>
-      </c>
-      <c r="B117" s="33" t="inlineStr">
-        <is>
-          <t>page_index\router.py</t>
-        </is>
-      </c>
-      <c r="C117" s="33" t="inlineStr">
-        <is>
-          <t>65</t>
-        </is>
-      </c>
-      <c r="D117" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E117" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F117" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="23.25" customHeight="1" s="25">
-      <c r="A118" s="34" t="n">
-        <v>117</v>
-      </c>
-      <c r="B118" s="34" t="inlineStr">
-        <is>
-          <t>plugins\router.py</t>
-        </is>
-      </c>
-      <c r="C118" s="34" t="inlineStr">
-        <is>
-          <t>267</t>
-        </is>
-      </c>
-      <c r="D118" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E118" s="34" t="inlineStr">
-        <is>
-          <t>Browse available plugins in the marketplace (placeholder for future implementati</t>
-        </is>
-      </c>
-      <c r="F118" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="119" ht="15" customHeight="1" s="25">
-      <c r="A119" s="34" t="n">
-        <v>118</v>
-      </c>
-      <c r="B119" s="34" t="inlineStr">
-        <is>
-          <t>plugins\router.py</t>
-        </is>
-      </c>
-      <c r="C119" s="34" t="inlineStr">
-        <is>
-          <t>269</t>
-        </is>
-      </c>
-      <c r="D119" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E119" s="34" t="inlineStr">
-        <is>
-          <t># This is a placeholder for future marketplace implementation</t>
-        </is>
-      </c>
-      <c r="F119" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="120" ht="15" customHeight="1" s="25">
-      <c r="A120" s="34" t="n">
-        <v>119</v>
-      </c>
-      <c r="B120" s="34" t="inlineStr">
-        <is>
-          <t>plugins\router.py</t>
-        </is>
-      </c>
-      <c r="C120" s="34" t="inlineStr">
-        <is>
-          <t>271</t>
-        </is>
-      </c>
-      <c r="D120" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E120" s="34" t="inlineStr">
-        <is>
-          <t>"message": "Plugin marketplace coming soon!",</t>
-        </is>
-      </c>
-      <c r="F120" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="121" ht="15" customHeight="1" s="25">
-      <c r="A121" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="B121" s="33" t="inlineStr">
-        <is>
-          <t>registry\router.py</t>
-        </is>
-      </c>
-      <c r="C121" s="33" t="inlineStr">
-        <is>
-          <t>271</t>
-        </is>
-      </c>
-      <c r="D121" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E121" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F121" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="122" ht="15" customHeight="1" s="25">
-      <c r="A122" s="33" t="n">
-        <v>121</v>
-      </c>
-      <c r="B122" s="33" t="inlineStr">
-        <is>
-          <t>registry\router.py</t>
-        </is>
-      </c>
-      <c r="C122" s="33" t="inlineStr">
-        <is>
-          <t>500</t>
-        </is>
-      </c>
-      <c r="D122" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E122" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F122" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="123" ht="15" customHeight="1" s="25">
-      <c r="A123" s="35" t="n">
-        <v>122</v>
-      </c>
-      <c r="B123" s="35" t="inlineStr">
-        <is>
-          <t>registry\router.py</t>
-        </is>
-      </c>
-      <c r="C123" s="35" t="inlineStr">
-        <is>
-          <t>628</t>
-        </is>
-      </c>
-      <c r="D123" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E123" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F123" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="15" customHeight="1" s="25">
-      <c r="A124" s="33" t="n">
-        <v>123</v>
-      </c>
-      <c r="B124" s="33" t="inlineStr">
-        <is>
-          <t>rent\router.py</t>
-        </is>
-      </c>
-      <c r="C124" s="33" t="inlineStr">
-        <is>
-          <t>310</t>
-        </is>
-      </c>
-      <c r="D124" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E124" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F124" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="15" customHeight="1" s="25">
-      <c r="A125" s="35" t="n">
-        <v>124</v>
-      </c>
-      <c r="B125" s="35" t="inlineStr">
-        <is>
-          <t>research\service.py</t>
-        </is>
-      </c>
-      <c r="C125" s="35" t="inlineStr">
-        <is>
-          <t>204</t>
-        </is>
-      </c>
-      <c r="D125" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E125" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F125" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="15" customHeight="1" s="25">
-      <c r="A126" s="35" t="n">
-        <v>125</v>
-      </c>
-      <c r="B126" s="35" t="inlineStr">
-        <is>
-          <t>research\service.py</t>
-        </is>
-      </c>
-      <c r="C126" s="35" t="inlineStr">
-        <is>
-          <t>353</t>
-        </is>
-      </c>
-      <c r="D126" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E126" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F126" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" ht="15" customHeight="1" s="25">
-      <c r="A127" s="34" t="n">
-        <v>126</v>
-      </c>
-      <c r="B127" s="34" t="inlineStr">
-        <is>
-          <t>role_upgrade\router.py</t>
-        </is>
-      </c>
-      <c r="C127" s="34" t="inlineStr">
-        <is>
-          <t>149</t>
-        </is>
-      </c>
-      <c r="D127" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E127" s="34" t="inlineStr">
-        <is>
-          <t># TEMPORARY: Professional roles coming soon (Q3 2026)</t>
-        </is>
-      </c>
-      <c r="F127" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" ht="15" customHeight="1" s="25">
-      <c r="A128" s="33" t="n">
-        <v>127</v>
-      </c>
-      <c r="B128" s="33" t="inlineStr">
-        <is>
-          <t>search\router.py</t>
-        </is>
-      </c>
-      <c r="C128" s="33" t="inlineStr">
-        <is>
-          <t>447</t>
-        </is>
-      </c>
-      <c r="D128" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E128" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F128" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" ht="15" customHeight="1" s="25">
-      <c r="A129" s="33" t="n">
-        <v>128</v>
-      </c>
-      <c r="B129" s="33" t="inlineStr">
-        <is>
-          <t>security\router.py</t>
-        </is>
-      </c>
-      <c r="C129" s="33" t="inlineStr">
-        <is>
-          <t>38</t>
-        </is>
-      </c>
-      <c r="D129" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E129" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F129" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="130" ht="15" customHeight="1" s="25">
-      <c r="A130" s="33" t="n">
-        <v>129</v>
-      </c>
-      <c r="B130" s="33" t="inlineStr">
-        <is>
-          <t>setup\router.py</t>
-        </is>
-      </c>
-      <c r="C130" s="33" t="inlineStr">
-        <is>
-          <t>327</t>
-        </is>
-      </c>
-      <c r="D130" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E130" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F130" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="131" ht="15" customHeight="1" s="25">
-      <c r="A131" s="34" t="n">
-        <v>130</v>
-      </c>
-      <c r="B131" s="34" t="inlineStr">
-        <is>
-          <t>storage\router.py</t>
-        </is>
-      </c>
-      <c r="C131" s="34" t="inlineStr">
-        <is>
-          <t>973</t>
-        </is>
-      </c>
-      <c r="D131" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E131" s="34" t="inlineStr">
-        <is>
-          <t>&lt;div class="provider-desc"&gt;Coming soon&lt;/div&gt;</t>
-        </is>
-      </c>
-      <c r="F131" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="132" ht="15" customHeight="1" s="25">
-      <c r="A132" s="33" t="n">
-        <v>131</v>
-      </c>
-      <c r="B132" s="33" t="inlineStr">
-        <is>
-          <t>storage\router.py</t>
-        </is>
-      </c>
-      <c r="C132" s="33" t="inlineStr">
-        <is>
-          <t>1602</t>
-        </is>
-      </c>
-      <c r="D132" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E132" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F132" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" ht="15" customHeight="1" s="25">
-      <c r="A133" s="33" t="n">
-        <v>132</v>
-      </c>
-      <c r="B133" s="33" t="inlineStr">
-        <is>
-          <t>storage\router.py</t>
-        </is>
-      </c>
-      <c r="C133" s="33" t="inlineStr">
-        <is>
-          <t>1605</t>
-        </is>
-      </c>
-      <c r="D133" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E133" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F133" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="134" ht="15" customHeight="1" s="25">
-      <c r="A134" s="33" t="n">
-        <v>133</v>
-      </c>
-      <c r="B134" s="33" t="inlineStr">
-        <is>
-          <t>tactics\router.py</t>
-        </is>
-      </c>
-      <c r="C134" s="33" t="inlineStr">
-        <is>
-          <t>128</t>
-        </is>
-      </c>
-      <c r="D134" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E134" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F134" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="15" customHeight="1" s="25">
-      <c r="A135" s="33" t="n">
-        <v>134</v>
-      </c>
-      <c r="B135" s="33" t="inlineStr">
-        <is>
-          <t>tenant_feed\service.py</t>
-        </is>
-      </c>
-      <c r="C135" s="33" t="inlineStr">
-        <is>
-          <t>319</t>
-        </is>
-      </c>
-      <c r="D135" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E135" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F135" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="136" ht="15" customHeight="1" s="25">
-      <c r="A136" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="B136" s="33" t="inlineStr">
-        <is>
-          <t>tenant_feed\service.py</t>
-        </is>
-      </c>
-      <c r="C136" s="33" t="inlineStr">
-        <is>
-          <t>351</t>
-        </is>
-      </c>
-      <c r="D136" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E136" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F136" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="137" ht="15" customHeight="1" s="25">
-      <c r="A137" s="33" t="n">
-        <v>136</v>
-      </c>
-      <c r="B137" s="33" t="inlineStr">
-        <is>
-          <t>tenant_feed\service.py</t>
-        </is>
-      </c>
-      <c r="C137" s="33" t="inlineStr">
-        <is>
-          <t>383</t>
-        </is>
-      </c>
-      <c r="D137" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E137" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F137" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="138" ht="15" customHeight="1" s="25">
-      <c r="A138" s="33" t="n">
-        <v>137</v>
-      </c>
-      <c r="B138" s="33" t="inlineStr">
-        <is>
-          <t>timeline\router.py</t>
-        </is>
-      </c>
-      <c r="C138" s="33" t="inlineStr">
-        <is>
-          <t>320</t>
-        </is>
-      </c>
-      <c r="D138" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E138" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F138" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="15" customHeight="1" s="25">
-      <c r="A139" s="33" t="n">
-        <v>138</v>
-      </c>
-      <c r="B139" s="33" t="inlineStr">
-        <is>
-          <t>timeline\router.py</t>
-        </is>
-      </c>
-      <c r="C139" s="33" t="inlineStr">
-        <is>
-          <t>393</t>
-        </is>
-      </c>
-      <c r="D139" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E139" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F139" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="15" customHeight="1" s="25">
-      <c r="A140" s="35" t="n">
-        <v>139</v>
-      </c>
-      <c r="B140" s="35" t="inlineStr">
-        <is>
-          <t>timeline\router.py</t>
-        </is>
-      </c>
-      <c r="C140" s="35" t="inlineStr">
-        <is>
-          <t>394</t>
-        </is>
-      </c>
-      <c r="D140" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E140" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F140" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="141" ht="15" customHeight="1" s="25">
-      <c r="A141" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="B141" s="33" t="inlineStr">
-        <is>
-          <t>timeline\router.py</t>
-        </is>
-      </c>
-      <c r="C141" s="33" t="inlineStr">
-        <is>
-          <t>880</t>
-        </is>
-      </c>
-      <c r="D141" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E141" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F141" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="142" ht="15" customHeight="1" s="25">
-      <c r="A142" s="33" t="n">
-        <v>141</v>
-      </c>
-      <c r="B142" s="33" t="inlineStr">
-        <is>
-          <t>user\router.py</t>
-        </is>
-      </c>
-      <c r="C142" s="33" t="inlineStr">
-        <is>
-          <t>150</t>
-        </is>
-      </c>
-      <c r="D142" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E142" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F142" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="143" ht="15" customHeight="1" s="25">
-      <c r="A143" s="33" t="n">
-        <v>142</v>
-      </c>
-      <c r="B143" s="33" t="inlineStr">
-        <is>
-          <t>vault\router.py</t>
-        </is>
-      </c>
-      <c r="C143" s="33" t="inlineStr">
-        <is>
-          <t>224</t>
-        </is>
-      </c>
-      <c r="D143" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E143" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F143" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="144" ht="15" customHeight="1" s="25">
-      <c r="A144" s="34" t="n">
-        <v>143</v>
-      </c>
-      <c r="B144" s="34" t="inlineStr">
-        <is>
-          <t>vault\router.py</t>
-        </is>
-      </c>
-      <c r="C144" s="34" t="inlineStr">
-        <is>
-          <t>300</t>
-        </is>
-      </c>
-      <c r="D144" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E144" s="34" t="inlineStr">
-        <is>
-          <t># Resolve real access token (form field may be "auto" placeholder from JS)</t>
-        </is>
-      </c>
-      <c r="F144" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="145" ht="15" customHeight="1" s="25">
-      <c r="A145" s="33" t="n">
-        <v>144</v>
-      </c>
-      <c r="B145" s="33" t="inlineStr">
-        <is>
-          <t>vault\router.py</t>
-        </is>
-      </c>
-      <c r="C145" s="33" t="inlineStr">
-        <is>
-          <t>309</t>
-        </is>
-      </c>
-      <c r="D145" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E145" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F145" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="146" ht="15" customHeight="1" s="25">
-      <c r="A146" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="B146" s="33" t="inlineStr">
-        <is>
-          <t>vault\router.py</t>
-        </is>
-      </c>
-      <c r="C146" s="33" t="inlineStr">
-        <is>
-          <t>1016</t>
-        </is>
-      </c>
-      <c r="D146" s="33" t="inlineStr">
-        <is>
-          <t>pass stub</t>
-        </is>
-      </c>
-      <c r="E146" s="33" t="inlineStr">
-        <is>
-          <t>Bare pass statement</t>
-        </is>
-      </c>
-      <c r="F146" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="147" ht="15" customHeight="1" s="25">
-      <c r="A147" s="35" t="n">
-        <v>146</v>
-      </c>
-      <c r="B147" s="35" t="inlineStr">
-        <is>
-          <t>workflow\router.py</t>
-        </is>
-      </c>
-      <c r="C147" s="35" t="inlineStr">
-        <is>
-          <t>284</t>
-        </is>
-      </c>
-      <c r="D147" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E147" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F147" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="148" ht="15" customHeight="1" s="25">
-      <c r="A148" s="35" t="n">
-        <v>147</v>
-      </c>
-      <c r="B148" s="35" t="inlineStr">
-        <is>
-          <t>workflow\router.py</t>
-        </is>
-      </c>
-      <c r="C148" s="35" t="inlineStr">
-        <is>
-          <t>308</t>
-        </is>
-      </c>
-      <c r="D148" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E148" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F148" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="149" ht="15" customHeight="1" s="25">
-      <c r="A149" s="33" t="n">
-        <v>148</v>
-      </c>
-      <c r="B149" s="33" t="inlineStr">
-        <is>
-          <t>_template\router.py</t>
-        </is>
-      </c>
-      <c r="C149" s="33" t="inlineStr">
-        <is>
-          <t>43</t>
-        </is>
-      </c>
-      <c r="D149" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E149" s="33" t="inlineStr">
-        <is>
-          <t># TODO: Replace with real list query</t>
-        </is>
-      </c>
-      <c r="F149" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="150" ht="15" customHeight="1" s="25">
-      <c r="A150" s="35" t="n">
-        <v>149</v>
-      </c>
-      <c r="B150" s="35" t="inlineStr">
-        <is>
-          <t>_template\router.py</t>
-        </is>
-      </c>
-      <c r="C150" s="35" t="inlineStr">
-        <is>
-          <t>44</t>
-        </is>
-      </c>
-      <c r="D150" s="35" t="inlineStr">
-        <is>
-          <t>empty return</t>
-        </is>
-      </c>
-      <c r="E150" s="35" t="inlineStr">
-        <is>
-          <t>Returns empty list/dict</t>
-        </is>
-      </c>
-      <c r="F150" s="35" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-    </row>
-    <row r="151" ht="15" customHeight="1" s="25">
-      <c r="A151" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="B151" s="33" t="inlineStr">
-        <is>
-          <t>_template\service.py</t>
-        </is>
-      </c>
-      <c r="C151" s="33" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="D151" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E151" s="33" t="inlineStr">
-        <is>
-          <t># TODO: Replace with real DB/storage lookup</t>
-        </is>
-      </c>
-      <c r="F151" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="152" ht="15" customHeight="1" s="25">
-      <c r="A152" s="33" t="n">
-        <v>151</v>
-      </c>
-      <c r="B152" s="33" t="inlineStr">
-        <is>
-          <t>_template\service.py</t>
-        </is>
-      </c>
-      <c r="C152" s="33" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="D152" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E152" s="33" t="inlineStr">
-        <is>
-          <t># TODO: Replace with real persistence</t>
-        </is>
-      </c>
-      <c r="F152" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="153" ht="15" customHeight="1" s="25">
-      <c r="A153" s="34" t="n">
-        <v>152</v>
-      </c>
-      <c r="B153" s="34" t="inlineStr">
-        <is>
-          <t>_template\service.py</t>
-        </is>
-      </c>
-      <c r="C153" s="34" t="inlineStr">
-        <is>
-          <t>27</t>
-        </is>
-      </c>
-      <c r="D153" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E153" s="34" t="inlineStr">
-        <is>
-          <t>"id": "placeholder-id",</t>
-        </is>
-      </c>
-      <c r="F153" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
-    <row r="154" ht="15" customHeight="1" s="25">
-      <c r="A154" s="33" t="n">
-        <v>153</v>
-      </c>
-      <c r="B154" s="33" t="inlineStr">
-        <is>
-          <t>_template\service.py</t>
-        </is>
-      </c>
-      <c r="C154" s="33" t="inlineStr">
-        <is>
-          <t>35</t>
-        </is>
-      </c>
-      <c r="D154" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E154" s="33" t="inlineStr">
-        <is>
-          <t># TODO: Replace with real update logic</t>
-        </is>
-      </c>
-      <c r="F154" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="155" ht="15" customHeight="1" s="25">
-      <c r="A155" s="33" t="n">
-        <v>154</v>
-      </c>
-      <c r="B155" s="33" t="inlineStr">
-        <is>
-          <t>_template\service.py</t>
-        </is>
-      </c>
-      <c r="C155" s="33" t="inlineStr">
-        <is>
-          <t>41</t>
-        </is>
-      </c>
-      <c r="D155" s="33" t="inlineStr">
-        <is>
-          <t>TODO/FIXME</t>
-        </is>
-      </c>
-      <c r="E155" s="33" t="inlineStr">
-        <is>
-          <t># TODO: Replace with real delete logic</t>
-        </is>
-      </c>
-      <c r="F155" s="33" t="inlineStr">
-        <is>
-          <t>MEDIUM</t>
-        </is>
-      </c>
-    </row>
-    <row r="156" ht="15" customHeight="1" s="25">
-      <c r="A156" s="34" t="n">
-        <v>155</v>
-      </c>
-      <c r="B156" s="34" t="inlineStr">
-        <is>
-          <t>_template\__init__.py</t>
-        </is>
-      </c>
-      <c r="C156" s="34" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="D156" s="34" t="inlineStr">
-        <is>
-          <t>placeholder</t>
-        </is>
-      </c>
-      <c r="E156" s="34" t="inlineStr">
-        <is>
-          <t>`app/modules/&lt;your_module&gt;/` and replace placeholders.</t>
-        </is>
-      </c>
-      <c r="F156" s="34" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-    </row>
+    <row r="2" ht="15" customHeight="1" s="25"/>
+    <row r="3" ht="15" customHeight="1" s="25"/>
+    <row r="4" ht="15" customHeight="1" s="25"/>
+    <row r="5" ht="15" customHeight="1" s="25"/>
+    <row r="6" ht="15" customHeight="1" s="25"/>
+    <row r="7" ht="15" customHeight="1" s="25"/>
+    <row r="8" ht="15" customHeight="1" s="25"/>
+    <row r="9" ht="15" customHeight="1" s="25"/>
+    <row r="10" ht="15" customHeight="1" s="25"/>
+    <row r="11" ht="15" customHeight="1" s="25"/>
+    <row r="12" ht="15" customHeight="1" s="25"/>
+    <row r="13" ht="15" customHeight="1" s="25"/>
+    <row r="14" ht="15" customHeight="1" s="25"/>
+    <row r="15" ht="15" customHeight="1" s="25"/>
+    <row r="16" ht="15" customHeight="1" s="25"/>
+    <row r="17" ht="15" customHeight="1" s="25"/>
+    <row r="18" ht="15" customHeight="1" s="25"/>
+    <row r="19" ht="15" customHeight="1" s="25"/>
+    <row r="20" ht="15" customHeight="1" s="25"/>
+    <row r="21" ht="15" customHeight="1" s="25"/>
+    <row r="22" ht="15" customHeight="1" s="25"/>
+    <row r="23" ht="15" customHeight="1" s="25"/>
+    <row r="24" ht="15" customHeight="1" s="25"/>
+    <row r="25" ht="15" customHeight="1" s="25"/>
+    <row r="26" ht="15" customHeight="1" s="25"/>
+    <row r="27" ht="15" customHeight="1" s="25"/>
+    <row r="28" ht="15" customHeight="1" s="25"/>
+    <row r="29" ht="15" customHeight="1" s="25"/>
+    <row r="30" ht="15" customHeight="1" s="25"/>
+    <row r="31" ht="15" customHeight="1" s="25"/>
+    <row r="32" ht="15" customHeight="1" s="25"/>
+    <row r="33" ht="15" customHeight="1" s="25"/>
+    <row r="34" ht="15" customHeight="1" s="25"/>
+    <row r="35" ht="15" customHeight="1" s="25"/>
+    <row r="36" ht="15" customHeight="1" s="25"/>
+    <row r="37" ht="15" customHeight="1" s="25"/>
+    <row r="38" ht="15" customHeight="1" s="25"/>
+    <row r="39" ht="15" customHeight="1" s="25"/>
+    <row r="40" ht="15" customHeight="1" s="25"/>
+    <row r="41" ht="15" customHeight="1" s="25"/>
+    <row r="42" ht="15" customHeight="1" s="25"/>
+    <row r="43" ht="15" customHeight="1" s="25"/>
+    <row r="44" ht="15" customHeight="1" s="25"/>
+    <row r="45" ht="15" customHeight="1" s="25"/>
+    <row r="46" ht="15" customHeight="1" s="25"/>
+    <row r="47" ht="15" customHeight="1" s="25"/>
+    <row r="48" ht="15" customHeight="1" s="25"/>
+    <row r="49" ht="15" customHeight="1" s="25"/>
+    <row r="50" ht="15" customHeight="1" s="25"/>
+    <row r="51" ht="15" customHeight="1" s="25"/>
+    <row r="52" ht="15" customHeight="1" s="25"/>
+    <row r="53" ht="15" customHeight="1" s="25"/>
+    <row r="54" ht="15" customHeight="1" s="25"/>
+    <row r="55" ht="15" customHeight="1" s="25"/>
+    <row r="56" ht="15" customHeight="1" s="25"/>
+    <row r="57" ht="15" customHeight="1" s="25"/>
+    <row r="58" ht="15" customHeight="1" s="25"/>
+    <row r="59" ht="15" customHeight="1" s="25"/>
+    <row r="60" ht="15" customHeight="1" s="25"/>
+    <row r="61" ht="15" customHeight="1" s="25"/>
+    <row r="62" ht="15" customHeight="1" s="25"/>
+    <row r="63" ht="15" customHeight="1" s="25"/>
+    <row r="64" ht="15" customHeight="1" s="25"/>
+    <row r="65" ht="15" customHeight="1" s="25"/>
+    <row r="66" ht="15" customHeight="1" s="25"/>
+    <row r="67" ht="15" customHeight="1" s="25"/>
+    <row r="68" ht="15" customHeight="1" s="25"/>
+    <row r="69" ht="15" customHeight="1" s="25"/>
+    <row r="70" ht="15" customHeight="1" s="25"/>
+    <row r="71" ht="15" customHeight="1" s="25"/>
+    <row r="72" ht="15" customHeight="1" s="25"/>
+    <row r="73" ht="15" customHeight="1" s="25"/>
+    <row r="74" ht="15" customHeight="1" s="25"/>
+    <row r="75" ht="15" customHeight="1" s="25"/>
+    <row r="76" ht="15" customHeight="1" s="25"/>
+    <row r="77" ht="15" customHeight="1" s="25"/>
+    <row r="78" ht="15" customHeight="1" s="25"/>
+    <row r="79" ht="15" customHeight="1" s="25"/>
+    <row r="80" ht="15" customHeight="1" s="25"/>
+    <row r="81" ht="15" customHeight="1" s="25"/>
+    <row r="82" ht="15" customHeight="1" s="25"/>
+    <row r="83" ht="15" customHeight="1" s="25"/>
+    <row r="84" ht="15" customHeight="1" s="25"/>
+    <row r="85" ht="15" customHeight="1" s="25"/>
+    <row r="86" ht="15" customHeight="1" s="25"/>
+    <row r="87" ht="15" customHeight="1" s="25"/>
+    <row r="88" ht="15" customHeight="1" s="25"/>
+    <row r="89" ht="15" customHeight="1" s="25"/>
+    <row r="90" ht="15" customHeight="1" s="25"/>
+    <row r="91" ht="15" customHeight="1" s="25"/>
+    <row r="92" ht="15" customHeight="1" s="25"/>
+    <row r="93" ht="15" customHeight="1" s="25"/>
+    <row r="94" ht="15" customHeight="1" s="25"/>
+    <row r="95" ht="15" customHeight="1" s="25"/>
+    <row r="96" ht="15" customHeight="1" s="25"/>
+    <row r="97" ht="15" customHeight="1" s="25"/>
+    <row r="98" ht="15" customHeight="1" s="25"/>
+    <row r="99" ht="23.25" customHeight="1" s="25"/>
+    <row r="100" ht="23.25" customHeight="1" s="25"/>
+    <row r="101" ht="23.25" customHeight="1" s="25"/>
+    <row r="102" ht="23.25" customHeight="1" s="25"/>
+    <row r="103" ht="15" customHeight="1" s="25"/>
+    <row r="104" ht="15" customHeight="1" s="25"/>
+    <row r="105" ht="15" customHeight="1" s="25"/>
+    <row r="106" ht="15" customHeight="1" s="25"/>
+    <row r="107" ht="15" customHeight="1" s="25"/>
+    <row r="108" ht="15" customHeight="1" s="25"/>
+    <row r="109" ht="15" customHeight="1" s="25"/>
+    <row r="110" ht="15" customHeight="1" s="25"/>
+    <row r="111" ht="23.25" customHeight="1" s="25"/>
+    <row r="112" ht="15" customHeight="1" s="25"/>
+    <row r="113" ht="15" customHeight="1" s="25"/>
+    <row r="114" ht="15" customHeight="1" s="25"/>
+    <row r="115" ht="23.25" customHeight="1" s="25"/>
+    <row r="116" ht="15" customHeight="1" s="25"/>
+    <row r="117" ht="15" customHeight="1" s="25"/>
+    <row r="118" ht="23.25" customHeight="1" s="25"/>
+    <row r="119" ht="15" customHeight="1" s="25"/>
+    <row r="120" ht="15" customHeight="1" s="25"/>
+    <row r="121" ht="15" customHeight="1" s="25"/>
+    <row r="122" ht="15" customHeight="1" s="25"/>
+    <row r="123" ht="15" customHeight="1" s="25"/>
+    <row r="124" ht="15" customHeight="1" s="25"/>
+    <row r="125" ht="15" customHeight="1" s="25"/>
+    <row r="126" ht="15" customHeight="1" s="25"/>
+    <row r="127" ht="15" customHeight="1" s="25"/>
+    <row r="128" ht="15" customHeight="1" s="25"/>
+    <row r="129" ht="15" customHeight="1" s="25"/>
+    <row r="130" ht="15" customHeight="1" s="25"/>
+    <row r="131" ht="15" customHeight="1" s="25"/>
+    <row r="132" ht="15" customHeight="1" s="25"/>
+    <row r="133" ht="15" customHeight="1" s="25"/>
+    <row r="134" ht="15" customHeight="1" s="25"/>
+    <row r="135" ht="15" customHeight="1" s="25"/>
+    <row r="136" ht="15" customHeight="1" s="25"/>
+    <row r="137" ht="15" customHeight="1" s="25"/>
+    <row r="138" ht="15" customHeight="1" s="25"/>
+    <row r="139" ht="15" customHeight="1" s="25"/>
+    <row r="140" ht="15" customHeight="1" s="25"/>
+    <row r="141" ht="15" customHeight="1" s="25"/>
+    <row r="142" ht="15" customHeight="1" s="25"/>
+    <row r="143" ht="15" customHeight="1" s="25"/>
+    <row r="144" ht="15" customHeight="1" s="25"/>
+    <row r="145" ht="15" customHeight="1" s="25"/>
+    <row r="146" ht="15" customHeight="1" s="25"/>
+    <row r="147" ht="15" customHeight="1" s="25"/>
+    <row r="148" ht="15" customHeight="1" s="25"/>
+    <row r="149" ht="15" customHeight="1" s="25"/>
+    <row r="150" ht="15" customHeight="1" s="25"/>
+    <row r="151" ht="15" customHeight="1" s="25"/>
+    <row r="152" ht="15" customHeight="1" s="25"/>
+    <row r="153" ht="15" customHeight="1" s="25"/>
+    <row r="154" ht="15" customHeight="1" s="25"/>
+    <row r="155" ht="15" customHeight="1" s="25"/>
+    <row r="156" ht="15" customHeight="1" s="25"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
fix(workbook_bridge): preserve manual Stubs & TODOs rows across sync
- tools/workbook_bridge.py: update_excel_stubs() now uses a Source marker column (G) to tag script-written rows as 'auto'. Hand-typed rows are preserved across syncs instead of being wiped. Added _log_stub_sync_to_build_state() to log before/after row counts to BUILD_STATE.md on every sync.
- BUILD_STATE.md: added session note and stub sync log section.
- Semptify_Master_Inventory_LIVE_reviewed.xlsx: Source header added to column G of Stubs & TODOs sheet.
- tools/agent_orchestrator_tasks.json: regenerated (16 tasks, no change to task data).
</commit_message>
<xml_diff>
--- a/Semptify_Master_Inventory_LIVE_reviewed.xlsx
+++ b/Semptify_Master_Inventory_LIVE_reviewed.xlsx
@@ -2399,7 +2399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="24" min="1" max="1"/>
@@ -2439,6 +2439,11 @@
       <c r="F1" s="31" t="inlineStr">
         <is>
           <t>Severity</t>
+        </is>
+      </c>
+      <c r="G1" s="24" t="inlineStr">
+        <is>
+          <t>Source</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore(orchestrator): archive 16 resolved duplicates; fix empty-queue bug in workbook_bridge
Ran archive_resolved_duplicates.py to move all 16 resolved duplicate-resolve rows from the 'Duplicates' sheet to the 'Archive' sheet in Semptify_Master_Inventory_LIVE_reviewed.xlsx. The active queue is now empty (0 tasks).

Also fix workbook_bridge.py: was treating '0 tasks generated' as a failure (exit 1). After archiving, an empty Duplicates sheet is the correct, expected state. Now writes the empty task list and returns 0 with a clear message.

Refreshed agent_orchestrator.html and orchestrator_dashboard.html embedded JSON via sync_orchestrator.py.
</commit_message>
<xml_diff>
--- a/Semptify_Master_Inventory_LIVE_reviewed.xlsx
+++ b/Semptify_Master_Inventory_LIVE_reviewed.xlsx
@@ -23,6 +23,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gap Check" sheetId="14" state="visible" r:id="rId14"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI Resource Roster" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Task Queue" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Archive" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -2615,7 +2616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="24" min="1" max="1"/>
@@ -2646,326 +2647,22 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="23.25" customHeight="1" s="25">
-      <c r="A2" s="33" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="33" t="inlineStr">
-        <is>
-          <t>vault vs vault_engine vs vault_all_in_one</t>
-        </is>
-      </c>
-      <c r="C2" s="33" t="inlineStr">
-        <is>
-          <t>3 vault modules with overlapping functionality</t>
-        </is>
-      </c>
-      <c r="D2" s="33" t="inlineStr">
-        <is>
-          <t>vault.router (17 routes), vault_engine.router (11 routes), vault_all_in_one.router (13 routes) — all deal with vault operations.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="23.25" customHeight="1" s="25">
-      <c r="A3" s="33" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="33" t="inlineStr">
-        <is>
-          <t>case_builder router vs case_builder.py standalone</t>
-        </is>
-      </c>
-      <c r="C3" s="33" t="inlineStr">
-        <is>
-          <t>Module router vs standalone file</t>
-        </is>
-      </c>
-      <c r="D3" s="33" t="inlineStr">
-        <is>
-          <t>app/modules/case_builder/router.py (36 routes) and app/modules/case_builder.py (27917 bytes). Standalone may be legacy.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="23.25" customHeight="1" s="25">
-      <c r="A4" s="33" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="33" t="inlineStr">
-        <is>
-          <t>document_converter router vs standalone</t>
-        </is>
-      </c>
-      <c r="C4" s="33" t="inlineStr">
-        <is>
-          <t>Module router vs standalone file</t>
-        </is>
-      </c>
-      <c r="D4" s="33" t="inlineStr">
-        <is>
-          <t>app/modules/document_converter/router.py (8 routes) and app/modules/document_converter.py (44828 bytes).</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="15" customHeight="1" s="25">
-      <c r="A5" s="33" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="33" t="inlineStr">
-        <is>
-          <t>research router vs research_module.py standalone</t>
-        </is>
-      </c>
-      <c r="C5" s="33" t="inlineStr">
-        <is>
-          <t>Module router vs standalone file</t>
-        </is>
-      </c>
-      <c r="D5" s="33" t="inlineStr">
-        <is>
-          <t>app/modules/research/router.py (18 routes) and app/modules/research_module.py (52568 bytes).</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="23.25" customHeight="1" s="25">
-      <c r="A6" s="33" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="33" t="inlineStr">
-        <is>
-          <t>tenant_defense vs eviction_defense</t>
-        </is>
-      </c>
-      <c r="C6" s="33" t="inlineStr">
-        <is>
-          <t>Overlapping domain</t>
-        </is>
-      </c>
-      <c r="D6" s="33" t="inlineStr">
-        <is>
-          <t>tenant_defense.py (11 endpoints) and eviction_defense/router.py (18 endpoints) — both deal with tenant defense.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1" s="25">
-      <c r="A7" s="33" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="33" t="inlineStr">
-        <is>
-          <t>complaints router vs complaint_wizard_module.py</t>
-        </is>
-      </c>
-      <c r="C7" s="33" t="inlineStr">
-        <is>
-          <t>Module router vs standalone file</t>
-        </is>
-      </c>
-      <c r="D7" s="33" t="inlineStr">
-        <is>
-          <t>complaints/router.py (18 routes) and complaint_wizard_module.py (24293 bytes, dev_only).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1" s="25">
-      <c r="A8" s="33" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="33" t="inlineStr">
-        <is>
-          <t>free_api router vs free_api_pack.py</t>
-        </is>
-      </c>
-      <c r="C8" s="33" t="inlineStr">
-        <is>
-          <t>Module router vs standalone file</t>
-        </is>
-      </c>
-      <c r="D8" s="33" t="inlineStr">
-        <is>
-          <t>free_api/router.py (11 routes) and free_api_pack.py (27681 bytes, dev_only).</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1" s="25">
-      <c r="A9" s="33" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="33" t="inlineStr">
-        <is>
-          <t>storage function-token/issue (duplicate route)</t>
-        </is>
-      </c>
-      <c r="C9" s="33" t="inlineStr">
-        <is>
-          <t>Duplicate route registration</t>
-        </is>
-      </c>
-      <c r="D9" s="33" t="inlineStr">
-        <is>
-          <t>storage/router.py registers POST /function-token/issue twice (lines 1003 and 1014).</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="15" customHeight="1" s="25">
-      <c r="A10" s="33" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="33" t="inlineStr">
-        <is>
-          <t>storage function-token/verify (duplicate route)</t>
-        </is>
-      </c>
-      <c r="C10" s="33" t="inlineStr">
-        <is>
-          <t>Duplicate route registration</t>
-        </is>
-      </c>
-      <c r="D10" s="33" t="inlineStr">
-        <is>
-          <t>storage/router.py registers POST /function-token/verify twice (lines 1004 and 1015).</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="15" customHeight="1" s="25">
-      <c r="A11" s="33" t="n">
-        <v>10</v>
-      </c>
-      <c r="B11" s="33" t="inlineStr">
-        <is>
-          <t>timeline vs briefcase timeline vs workflow timeline</t>
-        </is>
-      </c>
-      <c r="C11" s="33" t="inlineStr">
-        <is>
-          <t>3 timeline systems</t>
-        </is>
-      </c>
-      <c r="D11" s="33" t="inlineStr">
-        <is>
-          <t>timeline.router (3 routes), briefcase.router has 7 timeline-event routes, workflow has timeline logic.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="15" customHeight="1" s="25">
-      <c r="A12" s="33" t="n">
-        <v>11</v>
-      </c>
-      <c r="B12" s="33" t="inlineStr">
-        <is>
-          <t>cloud_sync vs user_cloud_sync service</t>
-        </is>
-      </c>
-      <c r="C12" s="33" t="inlineStr">
-        <is>
-          <t>Module vs service overlap</t>
-        </is>
-      </c>
-      <c r="D12" s="33" t="inlineStr">
-        <is>
-          <t>cloud_sync.router (19 routes) and services/user_cloud_sync.py (21881 bytes).</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="15" customHeight="1" s="25">
-      <c r="A13" s="33" t="n">
-        <v>12</v>
-      </c>
-      <c r="B13" s="33" t="inlineStr">
-        <is>
-          <t>search vs vault_search vs postgres_fts</t>
-        </is>
-      </c>
-      <c r="C13" s="33" t="inlineStr">
-        <is>
-          <t>3 search systems</t>
-        </is>
-      </c>
-      <c r="D13" s="33" t="inlineStr">
-        <is>
-          <t>search.router (7 routes), services/vault_search.py, core/postgres_fts.py.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="23.25" customHeight="1" s="25">
-      <c r="A14" s="33" t="n">
-        <v>13</v>
-      </c>
-      <c r="B14" s="33" t="inlineStr">
-        <is>
-          <t>brain vs positronic_brain vs positronic_mesh vs mesh_network</t>
-        </is>
-      </c>
-      <c r="C14" s="33" t="inlineStr">
-        <is>
-          <t>4 brain/mesh systems</t>
-        </is>
-      </c>
-      <c r="D14" s="33" t="inlineStr">
-        <is>
-          <t>brain.router (11), positronic_brain.py, positronic_mesh.router (13), mesh_network.router (11).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="15" customHeight="1" s="25">
-      <c r="A15" s="33" t="n">
-        <v>14</v>
-      </c>
-      <c r="B15" s="33" t="inlineStr">
-        <is>
-          <t>housing_accountability (0 routes in list)</t>
-        </is>
-      </c>
-      <c r="C15" s="33" t="inlineStr">
-        <is>
-          <t>Router exists but no routes listed</t>
-        </is>
-      </c>
-      <c r="D15" s="33" t="inlineStr">
-        <is>
-          <t>Registered in product_manifest but module_routes_list.txt shows 0 routes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="23.25" customHeight="1" s="25">
-      <c r="A16" s="33" t="n">
-        <v>15</v>
-      </c>
-      <c r="B16" s="33" t="inlineStr">
-        <is>
-          <t>litigation_intelligence (0 routes in list)</t>
-        </is>
-      </c>
-      <c r="C16" s="33" t="inlineStr">
-        <is>
-          <t>Router exists but no routes listed</t>
-        </is>
-      </c>
-      <c r="D16" s="33" t="inlineStr">
-        <is>
-          <t>Registered in product_manifest but module_routes_list.txt shows 0 routes. 17 endpoints claimed in ACTIVE_CONTEXT.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="15" customHeight="1" s="25">
-      <c r="A17" s="33" t="n">
-        <v>16</v>
-      </c>
-      <c r="B17" s="33" t="inlineStr">
-        <is>
-          <t>context_engine vs context_loop</t>
-        </is>
-      </c>
-      <c r="C17" s="33" t="inlineStr">
-        <is>
-          <t>Two context systems</t>
-        </is>
-      </c>
-      <c r="D17" s="33" t="inlineStr">
-        <is>
-          <t>context_engine.router (9 routes) and context_loop.router (11 routes) — both deal with context.</t>
-        </is>
-      </c>
-    </row>
+    <row r="2" ht="23.25" customHeight="1" s="25"/>
+    <row r="3" ht="23.25" customHeight="1" s="25"/>
+    <row r="4" ht="23.25" customHeight="1" s="25"/>
+    <row r="5" ht="15" customHeight="1" s="25"/>
+    <row r="6" ht="23.25" customHeight="1" s="25"/>
+    <row r="7" ht="15" customHeight="1" s="25"/>
+    <row r="8" ht="15" customHeight="1" s="25"/>
+    <row r="9" ht="15" customHeight="1" s="25"/>
+    <row r="10" ht="15" customHeight="1" s="25"/>
+    <row r="11" ht="15" customHeight="1" s="25"/>
+    <row r="12" ht="15" customHeight="1" s="25"/>
+    <row r="13" ht="15" customHeight="1" s="25"/>
+    <row r="14" ht="23.25" customHeight="1" s="25"/>
+    <row r="15" ht="15" customHeight="1" s="25"/>
+    <row r="16" ht="23.25" customHeight="1" s="25"/>
+    <row r="17" ht="15" customHeight="1" s="25"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -31888,6 +31585,532 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Systems</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Overlap Description</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Details/Notes</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Archived Status</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Archived Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>vault vs vault_engine vs vault_all_in_one</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>3 vault modules with overlapping functionality</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>vault.router (17 routes), vault_engine.router (11 routes), vault_all_in_one.router (13 routes) — all deal with vault operations.</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>case_builder router vs case_builder.py standalone</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Module router vs standalone file</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>app/modules/case_builder/router.py (36 routes) and app/modules/case_builder.py (27917 bytes). Standalone may be legacy.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>document_converter router vs standalone</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Module router vs standalone file</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>app/modules/document_converter/router.py (8 routes) and app/modules/document_converter.py (44828 bytes).</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>research router vs research_module.py standalone</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Module router vs standalone file</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>app/modules/research/router.py (18 routes) and app/modules/research_module.py (52568 bytes).</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>tenant_defense vs eviction_defense</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Overlapping domain</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>tenant_defense.py (11 endpoints) and eviction_defense/router.py (18 endpoints) — both deal with tenant defense.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>complaints router vs complaint_wizard_module.py</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Module router vs standalone file</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>complaints/router.py (18 routes) and complaint_wizard_module.py (24293 bytes, dev_only).</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>free_api router vs free_api_pack.py</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Module router vs standalone file</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>free_api/router.py (11 routes) and free_api_pack.py (27681 bytes, dev_only).</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>storage function-token/issue (duplicate route)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Duplicate route registration</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>storage/router.py registers POST /function-token/issue twice (lines 1003 and 1014).</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>storage function-token/verify (duplicate route)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Duplicate route registration</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>storage/router.py registers POST /function-token/verify twice (lines 1004 and 1015).</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>timeline vs briefcase timeline vs workflow timeline</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>3 timeline systems</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>timeline.router (3 routes), briefcase.router has 7 timeline-event routes, workflow has timeline logic.</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>cloud_sync vs user_cloud_sync service</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Module vs service overlap</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>cloud_sync.router (19 routes) and services/user_cloud_sync.py (21881 bytes).</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>search vs vault_search vs postgres_fts</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>3 search systems</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>search.router (7 routes), services/vault_search.py, core/postgres_fts.py.</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>brain vs positronic_brain vs positronic_mesh vs mesh_network</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>4 brain/mesh systems</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>brain.router (11), positronic_brain.py, positronic_mesh.router (13), mesh_network.router (11).</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>housing_accountability (0 routes in list)</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Router exists but no routes listed</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Registered in product_manifest but module_routes_list.txt shows 0 routes.</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>litigation_intelligence (0 routes in list)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Router exists but no routes listed</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Registered in product_manifest but module_routes_list.txt shows 0 routes. 17 endpoints claimed in ACTIVE_CONTEXT.</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>context_engine vs context_loop</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Two context systems</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>context_engine.router (9 routes) and context_loop.router (11 routes) — both deal with context.</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>resolved</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>2026-07-16T12:50:35.930301+00:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="0">

</xml_diff>